<commit_message>
Authorization page setup done
</commit_message>
<xml_diff>
--- a/cypress/fixtures/credentials.xlsx
+++ b/cypress/fixtures/credentials.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mostafizur\Desktop\Cypress\cypress\fixtures\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://leadscorp-my.sharepoint.com/personal/mostafizur_leads-bd_com/Documents/Desktop/Cypress Automation/MicroCube/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FBC05AD-2DBE-4CC7-83EE-7AEED75E2EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{0FBC05AD-2DBE-4CC7-83EE-7AEED75E2EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5090169A-CC50-4256-A7AB-4AA5090D71FD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,13 +30,13 @@
     <t>password</t>
   </si>
   <si>
-    <t>nusrat1</t>
-  </si>
-  <si>
     <t>username</t>
   </si>
   <si>
     <t>saikat</t>
+  </si>
+  <si>
+    <t>avisheak</t>
   </si>
 </sst>
 </file>
@@ -465,7 +465,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
@@ -473,7 +473,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
@@ -481,7 +481,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>

</xml_diff>

<commit_message>
url updated; read from excel implemented
</commit_message>
<xml_diff>
--- a/cypress/fixtures/credentials.xlsx
+++ b/cypress/fixtures/credentials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://leadscorp-my.sharepoint.com/personal/mostafizur_leads-bd_com/Documents/Desktop/Cypress Automation/MicroCube/cypress/fixtures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://leadscorp-my.sharepoint.com/personal/mostafizur_leads-bd_com/Documents/Desktop/Cypress Automation/SwiftFusion_Automation/cypress/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{0FBC05AD-2DBE-4CC7-83EE-7AEED75E2EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5090169A-CC50-4256-A7AB-4AA5090D71FD}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{0FBC05AD-2DBE-4CC7-83EE-7AEED75E2EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D420F70-EE7B-4EEE-A05B-CB278B2103EB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login_credentials" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>password</t>
   </si>
@@ -33,20 +33,31 @@
     <t>username</t>
   </si>
   <si>
-    <t>saikat</t>
+    <t>avisheak</t>
   </si>
   <si>
-    <t>avisheak</t>
+    <t>url</t>
+  </si>
+  <si>
+    <t>https://192.168.10.253:4941/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -153,10 +164,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -176,8 +188,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -456,38 +472,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="5"/>
-    <col min="2" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="25.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>3</v>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>4</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1">
-        <v>1</v>
-      </c>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{4772BE3F-FC0C-43AD-990E-DAE6636312E6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>